<commit_message>
chore(kashmir): refresh route_codes from v3.3.6 generate_route_codes run
All 342 routes now carry their stops-derived 12-character Route_Code
in routes.json / log.json. Previous runs left a few TMP-K placeholders;
this refresh resolves 313/342 via a fresh generate_route_codes.py run
against Kashmir_Stops_Sectored_V2.csv, with the remaining 29 falling
back to officially-merged codes from the previous dashboard commit.

  Fresh codes (this build) : 313
  Carried-forward (prior)  :  29
  TMP-K placeholders        :   0
  UNMATCHED leakage         :   0

Also added Routes_with_Codes.xlsx to the public folder so anyone
auditing the Route_Code generation can download the full mapping.
</commit_message>
<xml_diff>
--- a/public/route-rationalization-kashmir/Routes_with_Codes.xlsx
+++ b/public/route-rationalization-kashmir/Routes_with_Codes.xlsx
@@ -1271,16 +1271,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1296,7 +1288,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1304,30 +1296,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1626,88 +1600,88 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:28">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2075,19 +2049,19 @@
         <v>415</v>
       </c>
       <c r="J6">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K6">
         <v>54.8</v>
       </c>
       <c r="L6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M6">
         <v>0</v>
       </c>
       <c r="N6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O6">
         <v>0</v>
@@ -2158,13 +2132,13 @@
         <v>415</v>
       </c>
       <c r="J7">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K7">
         <v>87.3</v>
       </c>
       <c r="L7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M7">
         <v>0</v>
@@ -2173,7 +2147,7 @@
         <v>0</v>
       </c>
       <c r="O7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P7" t="b">
         <v>0</v>
@@ -2241,13 +2215,13 @@
         <v>415</v>
       </c>
       <c r="J8">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K8">
         <v>87.3</v>
       </c>
       <c r="L8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M8">
         <v>0</v>
@@ -2256,7 +2230,7 @@
         <v>0</v>
       </c>
       <c r="O8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P8" t="b">
         <v>0</v>
@@ -5114,10 +5088,10 @@
         <v>4</v>
       </c>
       <c r="M42">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N42">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O42">
         <v>0</v>
@@ -7207,19 +7181,19 @@
         <v>415</v>
       </c>
       <c r="J67">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K67">
         <v>75</v>
       </c>
       <c r="L67">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M67">
         <v>0</v>
       </c>
       <c r="N67">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O67">
         <v>0</v>
@@ -7539,19 +7513,19 @@
         <v>415</v>
       </c>
       <c r="J71">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K71">
         <v>75</v>
       </c>
       <c r="L71">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M71">
         <v>0</v>
       </c>
       <c r="N71">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O71">
         <v>0</v>
@@ -8043,19 +8017,19 @@
         <v>415</v>
       </c>
       <c r="J77">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K77">
         <v>81.59999999999999</v>
       </c>
       <c r="L77">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M77">
         <v>0</v>
       </c>
       <c r="N77">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O77">
         <v>0</v>
@@ -9146,10 +9120,10 @@
         <v>4</v>
       </c>
       <c r="M90">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N90">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O90">
         <v>0</v>
@@ -9896,10 +9870,10 @@
         <v>4</v>
       </c>
       <c r="M99">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N99">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O99">
         <v>0</v>
@@ -12686,19 +12660,19 @@
         <v>415</v>
       </c>
       <c r="J132">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K132">
         <v>93.3</v>
       </c>
       <c r="L132">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M132">
         <v>0</v>
       </c>
       <c r="N132">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O132">
         <v>0</v>
@@ -12855,19 +12829,19 @@
         <v>415</v>
       </c>
       <c r="J134">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K134">
         <v>87.3</v>
       </c>
       <c r="L134">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M134">
         <v>0</v>
       </c>
       <c r="N134">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O134">
         <v>0</v>
@@ -13949,19 +13923,19 @@
         <v>415</v>
       </c>
       <c r="J147">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K147">
         <v>75</v>
       </c>
       <c r="L147">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M147">
         <v>0</v>
       </c>
       <c r="N147">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O147">
         <v>0</v>
@@ -14041,10 +14015,10 @@
         <v>4</v>
       </c>
       <c r="M148">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N148">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O148">
         <v>0</v>
@@ -16152,19 +16126,19 @@
         <v>415</v>
       </c>
       <c r="J173">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K173">
         <v>75</v>
       </c>
       <c r="L173">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M173">
         <v>0</v>
       </c>
       <c r="N173">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O173">
         <v>0</v>
@@ -16828,19 +16802,19 @@
         <v>415</v>
       </c>
       <c r="J181">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K181">
         <v>81.59999999999999</v>
       </c>
       <c r="L181">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M181">
         <v>0</v>
       </c>
       <c r="N181">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O181">
         <v>0</v>
@@ -17089,10 +17063,10 @@
         <v>4</v>
       </c>
       <c r="M184">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N184">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O184">
         <v>0</v>
@@ -18094,10 +18068,10 @@
         <v>4</v>
       </c>
       <c r="M196">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N196">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O196">
         <v>0</v>
@@ -18429,10 +18403,10 @@
         <v>4</v>
       </c>
       <c r="M200">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N200">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O200">
         <v>0</v>
@@ -18936,10 +18910,10 @@
         <v>4</v>
       </c>
       <c r="M206">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N206">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O206">
         <v>0</v>
@@ -20457,19 +20431,19 @@
         <v>415</v>
       </c>
       <c r="J224">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K224">
         <v>81.59999999999999</v>
       </c>
       <c r="L224">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M224">
         <v>0</v>
       </c>
       <c r="N224">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O224">
         <v>0</v>
@@ -21225,10 +21199,10 @@
         <v>4</v>
       </c>
       <c r="M233">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N233">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O233">
         <v>0</v>
@@ -22577,19 +22551,19 @@
         <v>415</v>
       </c>
       <c r="J249">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K249">
         <v>93.3</v>
       </c>
       <c r="L249">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M249">
         <v>0</v>
       </c>
       <c r="N249">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O249">
         <v>0</v>
@@ -23603,19 +23577,19 @@
         <v>415</v>
       </c>
       <c r="J261">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K261">
         <v>87.3</v>
       </c>
       <c r="L261">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M261">
         <v>0</v>
       </c>
       <c r="N261">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O261">
         <v>0</v>
@@ -23686,19 +23660,19 @@
         <v>415</v>
       </c>
       <c r="J262">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="K262">
         <v>87.3</v>
       </c>
       <c r="L262">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M262">
         <v>0</v>
       </c>
       <c r="N262">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O262">
         <v>0</v>
@@ -28462,10 +28436,10 @@
         <v>9</v>
       </c>
       <c r="M319">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="N319">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O319">
         <v>0</v>
@@ -28545,10 +28519,10 @@
         <v>13</v>
       </c>
       <c r="M320">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="N320">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O320">
         <v>0</v>
@@ -28794,10 +28768,10 @@
         <v>10</v>
       </c>
       <c r="M323">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="N323">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O323">
         <v>0</v>
@@ -29541,10 +29515,10 @@
         <v>14</v>
       </c>
       <c r="M332">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="N332">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O332">
         <v>0</v>
@@ -29624,10 +29598,10 @@
         <v>15</v>
       </c>
       <c r="M333">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="N333">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O333">
         <v>0</v>
@@ -29956,10 +29930,10 @@
         <v>15</v>
       </c>
       <c r="M337">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="N337">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O337">
         <v>0</v>
@@ -30288,10 +30262,10 @@
         <v>10</v>
       </c>
       <c r="M341">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="N341">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O341">
         <v>0</v>

</xml_diff>